<commit_message>
fix(demo): simplify question_text to remove duplication in exam dashboard list
</commit_message>
<xml_diff>
--- a/Demo_Questions_Import.xlsx
+++ b/Demo_Questions_Import.xlsx
@@ -501,9 +501,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Find the largest of three numbers.
-Problem Description:
-Find the largest of three numbers.</t>
+          <t>Find the largest of three numbers.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -583,9 +581,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Write a function to check whether a number is prime.
-Problem Description:
-Write a function to check whether a number is prime.</t>
+          <t>Write a function to check whether a number is prime.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -665,9 +661,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Write a program to write data into a file and read it back.
-Problem Description:
-Write a program to write data into a file and read it back.</t>
+          <t>Write a program to write data into a file and read it back.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>